<commit_message>
Implement sample equity research report
</commit_message>
<xml_diff>
--- a/examples/family_bank_kenya/Family_Bank_Kenya_Financial_Model.xlsx
+++ b/examples/family_bank_kenya/Family_Bank_Kenya_Financial_Model.xlsx
@@ -13,6 +13,7 @@
     <sheet name="Scenarios" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="Model" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="Output" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Sources" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Area" localSheetId="0">'Cover'!$A$1:$J$29</definedName>
@@ -26,6 +27,7 @@
     <definedName name="_xlnm.Print_Area" localSheetId="4">'Model'!$B$1:$O$12,'Model'!$B$13:$O$101,'Model'!$B$102:$O$125,'Model'!$B$126:$O$142,'Model'!$B$143:$O$209,'Model'!$B$210:$O$240</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="5">'Output'!$1:$1</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="5">'Output'!$B$1:$O$84</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="6">'Sources'!$A$1:$G$19</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -312,7 +314,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="109">
+  <cellXfs count="114">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -619,6 +621,21 @@
     </xf>
     <xf numFmtId="2" fontId="12" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1514,7 +1531,11 @@
       <c r="A24" s="1" t="n"/>
       <c r="B24" s="1" t="n"/>
       <c r="C24" s="1" t="n"/>
-      <c r="D24" s="1" t="n"/>
+      <c r="D24" s="7" t="inlineStr">
+        <is>
+          <t>•  Sources (external market-data references)</t>
+        </is>
+      </c>
       <c r="E24" s="1" t="n"/>
       <c r="F24" s="1" t="n"/>
       <c r="G24" s="1" t="n"/>
@@ -15742,4 +15763,427 @@
     <firstFooter/>
   </headerFooter>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:P19"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="2" customWidth="1" min="1" max="1"/>
+    <col width="2" customWidth="1" min="2" max="2"/>
+    <col width="4" customWidth="1" min="3" max="3"/>
+    <col width="62" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="40" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="4" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="18" customHeight="1">
+      <c r="A1" s="11" t="n"/>
+      <c r="B1" s="11" t="n"/>
+      <c r="C1" s="12" t="inlineStr">
+        <is>
+          <t>FAMILY BANK LIMITED — DATA SOURCES &amp; REFERENCES</t>
+        </is>
+      </c>
+      <c r="H1" s="11" t="n"/>
+      <c r="I1" s="11" t="n"/>
+      <c r="J1" s="11" t="n"/>
+      <c r="K1" s="11" t="n"/>
+      <c r="L1" s="11" t="n"/>
+      <c r="M1" s="11" t="n"/>
+      <c r="N1" s="11" t="n"/>
+      <c r="O1" s="11" t="n"/>
+      <c r="P1" s="11" t="n"/>
+    </row>
+    <row r="2" ht="28" customHeight="1">
+      <c r="C2" s="109" t="inlineStr">
+        <is>
+          <t>Third-party market data used in this model's Output-sheet valuation (CAPM inputs, peer bank P/B multiples). Family Bank's own audited financial-statement figures are cited separately via research_output.md and the Assumptions sheet's data-provenance color legend.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="15" customHeight="1">
+      <c r="A4" s="11" t="n"/>
+      <c r="B4" s="11" t="n"/>
+      <c r="C4" s="83" t="inlineStr">
+        <is>
+          <t>REFERENCES</t>
+        </is>
+      </c>
+      <c r="D4" s="11" t="n"/>
+      <c r="E4" s="11" t="n"/>
+      <c r="F4" s="11" t="n"/>
+      <c r="G4" s="11" t="n"/>
+      <c r="H4" s="11" t="n"/>
+      <c r="I4" s="11" t="n"/>
+      <c r="J4" s="11" t="n"/>
+      <c r="K4" s="11" t="n"/>
+      <c r="L4" s="11" t="n"/>
+      <c r="M4" s="11" t="n"/>
+      <c r="N4" s="11" t="n"/>
+      <c r="O4" s="11" t="n"/>
+      <c r="P4" s="11" t="n"/>
+    </row>
+    <row r="5">
+      <c r="C5" s="32" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="D5" s="32" t="inlineStr">
+        <is>
+          <t>Item / Value</t>
+        </is>
+      </c>
+      <c r="E5" s="110" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+      <c r="F5" s="32" t="inlineStr">
+        <is>
+          <t>Source</t>
+        </is>
+      </c>
+      <c r="G5" s="110" t="inlineStr">
+        <is>
+          <t>Accessed</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="26" customHeight="1">
+      <c r="C6" s="10" t="inlineStr">
+        <is>
+          <t>[1]</t>
+        </is>
+      </c>
+      <c r="D6" s="111" t="inlineStr">
+        <is>
+          <t>Risk-free rate — Kenya 10-Year Government Bond Yield</t>
+        </is>
+      </c>
+      <c r="E6" s="112" t="inlineStr">
+        <is>
+          <t>12.32%</t>
+        </is>
+      </c>
+      <c r="F6" s="113">
+        <f>HYPERLINK("https://tradingeconomics.com/kenya/government-bond-yield","Trading Economics")</f>
+        <v/>
+      </c>
+      <c r="G6" s="112" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="26" customHeight="1">
+      <c r="C7" s="10" t="inlineStr">
+        <is>
+          <t>[2]</t>
+        </is>
+      </c>
+      <c r="D7" s="111" t="inlineStr">
+        <is>
+          <t>Equity risk premium — Kenya (total: mature-market ERP + country risk premium)</t>
+        </is>
+      </c>
+      <c r="E7" s="112" t="inlineStr">
+        <is>
+          <t>13.94%</t>
+        </is>
+      </c>
+      <c r="F7" s="113">
+        <f>HYPERLINK("https://pages.stern.nyu.edu/~adamodar/New_Home_Page/datafile/ctryprem.html","Aswath Damodaran, 'Country Default Spreads and Risk Premiums' (NYU Stern, Jan 2026 data update)")</f>
+        <v/>
+      </c>
+      <c r="G7" s="112" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="26" customHeight="1">
+      <c r="C8" s="10" t="inlineStr">
+        <is>
+          <t>[3]</t>
+        </is>
+      </c>
+      <c r="D8" s="111" t="inlineStr">
+        <is>
+          <t>Beta — average of 6 NSE-listed Kenyan peer bank equity betas (Absa 0.44, Co-op 0.52, DTB 0.28, Equity Group 0.59, I&amp;M 0.80, KCB 0.66)</t>
+        </is>
+      </c>
+      <c r="E8" s="112" t="inlineStr">
+        <is>
+          <t>0.55</t>
+        </is>
+      </c>
+      <c r="F8" s="113">
+        <f>HYPERLINK("https://live.mystocks.co.ke/","MyStocks Kenya")</f>
+        <v/>
+      </c>
+      <c r="G8" s="112" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="26" customHeight="1">
+      <c r="C9" s="10" t="inlineStr">
+        <is>
+          <t>[4]</t>
+        </is>
+      </c>
+      <c r="D9" s="111" t="inlineStr">
+        <is>
+          <t>Absa Bank Kenya — Price/Book (BVPS 19.58, share price 33.00)</t>
+        </is>
+      </c>
+      <c r="E9" s="112" t="inlineStr">
+        <is>
+          <t>1.69x</t>
+        </is>
+      </c>
+      <c r="F9" s="113">
+        <f>HYPERLINK("https://stockanalysis.com/","StockAnalysis.com")</f>
+        <v/>
+      </c>
+      <c r="G9" s="112" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="26" customHeight="1">
+      <c r="C10" s="10" t="inlineStr">
+        <is>
+          <t>[5]</t>
+        </is>
+      </c>
+      <c r="D10" s="111" t="inlineStr">
+        <is>
+          <t>Co-operative Bank of Kenya — Price/Book (BVPS 29.61, share price 35.00)</t>
+        </is>
+      </c>
+      <c r="E10" s="112" t="inlineStr">
+        <is>
+          <t>1.18x</t>
+        </is>
+      </c>
+      <c r="F10" s="113">
+        <f>HYPERLINK("https://stockanalysis.com/","StockAnalysis.com")</f>
+        <v/>
+      </c>
+      <c r="G10" s="112" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="26" customHeight="1">
+      <c r="C11" s="10" t="inlineStr">
+        <is>
+          <t>[6]</t>
+        </is>
+      </c>
+      <c r="D11" s="111" t="inlineStr">
+        <is>
+          <t>Diamond Trust Bank (DTB, ticker DTK) — Price/Book (BVPS 377.77, share price 150.75)</t>
+        </is>
+      </c>
+      <c r="E11" s="112" t="inlineStr">
+        <is>
+          <t>0.36x</t>
+        </is>
+      </c>
+      <c r="F11" s="113">
+        <f>HYPERLINK("https://stockanalysis.com/quote/nase/DTK/statistics/","StockAnalysis.com")</f>
+        <v/>
+      </c>
+      <c r="G11" s="112" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="26" customHeight="1">
+      <c r="C12" s="10" t="inlineStr">
+        <is>
+          <t>[7]</t>
+        </is>
+      </c>
+      <c r="D12" s="111" t="inlineStr">
+        <is>
+          <t>Equity Group Holdings — Price/Book (BVPS 86.57, share price 87.00)</t>
+        </is>
+      </c>
+      <c r="E12" s="112" t="inlineStr">
+        <is>
+          <t>0.96x</t>
+        </is>
+      </c>
+      <c r="F12" s="113">
+        <f>HYPERLINK("https://stockanalysis.com/","StockAnalysis.com")</f>
+        <v/>
+      </c>
+      <c r="G12" s="112" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="26" customHeight="1">
+      <c r="C13" s="10" t="inlineStr">
+        <is>
+          <t>[8]</t>
+        </is>
+      </c>
+      <c r="D13" s="111" t="inlineStr">
+        <is>
+          <t>I&amp;M Group — Price/Book (Book Value Per Share KES 66; share price ~42.50, company chart)</t>
+        </is>
+      </c>
+      <c r="E13" s="112" t="inlineStr">
+        <is>
+          <t>0.64x</t>
+        </is>
+      </c>
+      <c r="F13" s="30" t="inlineStr">
+        <is>
+          <t>I&amp;M Group FY2025 Integrated Report, p.120</t>
+        </is>
+      </c>
+      <c r="G13" s="112" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="26" customHeight="1">
+      <c r="C14" s="10" t="inlineStr">
+        <is>
+          <t>[9]</t>
+        </is>
+      </c>
+      <c r="D14" s="111" t="inlineStr">
+        <is>
+          <t>KCB Group — Price/Book (BVPS 109.61, share price 82.50)</t>
+        </is>
+      </c>
+      <c r="E14" s="112" t="inlineStr">
+        <is>
+          <t>0.73x</t>
+        </is>
+      </c>
+      <c r="F14" s="113">
+        <f>HYPERLINK("https://stockanalysis.com/","StockAnalysis.com")</f>
+        <v/>
+      </c>
+      <c r="G14" s="112" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="26" customHeight="1">
+      <c r="C15" s="10" t="inlineStr">
+        <is>
+          <t>[10]</t>
+        </is>
+      </c>
+      <c r="D15" s="111" t="inlineStr">
+        <is>
+          <t>NCBA Group — Price/Book (directly disclosed)</t>
+        </is>
+      </c>
+      <c r="E15" s="112" t="inlineStr">
+        <is>
+          <t>1.2x</t>
+        </is>
+      </c>
+      <c r="F15" s="30" t="inlineStr">
+        <is>
+          <t>NCBA Group Plc FY2025 Annual Integrated Report, p.32</t>
+        </is>
+      </c>
+      <c r="G15" s="112" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="26" customHeight="1">
+      <c r="C16" s="10" t="inlineStr">
+        <is>
+          <t>[11]</t>
+        </is>
+      </c>
+      <c r="D16" s="111" t="inlineStr">
+        <is>
+          <t>Stanbic Holdings — Price/Book (BVPS 202.74, share price 292.00)</t>
+        </is>
+      </c>
+      <c r="E16" s="112" t="inlineStr">
+        <is>
+          <t>1.44x</t>
+        </is>
+      </c>
+      <c r="F16" s="113">
+        <f>HYPERLINK("https://stockanalysis.com/","StockAnalysis.com")</f>
+        <v/>
+      </c>
+      <c r="G16" s="112" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="26" customHeight="1">
+      <c r="C17" s="10" t="inlineStr">
+        <is>
+          <t>[12]</t>
+        </is>
+      </c>
+      <c r="D17" s="111" t="inlineStr">
+        <is>
+          <t>Standard Chartered Bank Kenya (ticker SCBK) — Price/Book (BVPS 184.79, share price 334.25)</t>
+        </is>
+      </c>
+      <c r="E17" s="112" t="inlineStr">
+        <is>
+          <t>1.81x</t>
+        </is>
+      </c>
+      <c r="F17" s="113">
+        <f>HYPERLINK("https://stockanalysis.com/quote/nase/SCBK/statistics/","StockAnalysis.com")</f>
+        <v/>
+      </c>
+      <c r="G17" s="112" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="C19" s="109" t="inlineStr">
+        <is>
+          <t>Convention: Item/Value cited, Source (publisher — hyperlinked where a URL is available), Accessed (date the figure was pulled). Matches standard equity-research citation practice — see research_output.md for the full research log behind each entry.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="C1:G1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape"/>
+</worksheet>
 </file>
</xml_diff>